<commit_message>
Actualización plantillas Cuentas de AutDeRei y PagDeRei
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/AutDeRei-CuentasCuentasSeguidas.xlsx
+++ b/public/CuentasCuentas/AutDeRei-CuentasCuentasSeguidas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\CuentasCuentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732E9A8E-3302-4E36-BBB2-1B27CDC2BF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7A7D6A-9EE1-48A2-A4F7-0CE2578BFDAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="21">
   <si>
     <t>cuenta</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>3.2.2.1.01.01</t>
+  </si>
+  <si>
+    <t>Por la autorización del reintegro a la Tesorería de ingresos de aportaciones, en términos de las disposiciones aplicables</t>
   </si>
 </sst>
 </file>
@@ -652,7 +655,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
         <v>9</v>
@@ -666,7 +669,7 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
@@ -680,7 +683,7 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
         <v>9</v>
@@ -694,7 +697,7 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -708,7 +711,7 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D18" t="s">
         <v>9</v>
@@ -722,7 +725,7 @@
         <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D19" t="s">
         <v>4</v>
@@ -736,7 +739,7 @@
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D20" t="s">
         <v>9</v>
@@ -750,7 +753,7 @@
         <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -764,7 +767,7 @@
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
         <v>9</v>
@@ -778,7 +781,7 @@
         <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -792,7 +795,7 @@
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D24" t="s">
         <v>9</v>
@@ -806,7 +809,7 @@
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D25" t="s">
         <v>4</v>

</xml_diff>